<commit_message>
Finalize unified reporting workflows
</commit_message>
<xml_diff>
--- a/final/Excel/MVA_CrowdStrike_Final_Report.xlsx
+++ b/final/Excel/MVA_CrowdStrike_Final_Report.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R674dcd0a08cc4d7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="Rb7e7139243e44fcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="Rf1fd88f624104ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="Rf5819292cd5d4633"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="R04534b11f3254dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="R2f3a99e5239f49be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1377,7 +1377,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Discovered Vulnerabilities - Last 3 Months</a:t>
+              <a:t>Vulnerabilities Discovered</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1487,6 +1487,127 @@
 </file>
 
 <file path=xl/drawings/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>Vulnerabilities Remediated</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Remediated</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="70AD47"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Monthly Dashboard'!$A$11:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Monthly Dashboard'!$C$11:$C$13</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="30"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1629,7 +1750,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2a8519470dd402f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5a58a256c6be4a33"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1659,7 +1780,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R37188d9774c84e6b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b69d487e8fd429f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1689,7 +1810,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdac270d4f4fd44af"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R95c39958b6394b58"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1702,13 +1823,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1724,7 +1845,37 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6586b49a59e4dfe"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R180c710a43e74686"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rae89106a3a7e447a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1759,7 +1910,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb5ef71c409e4b7a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R207f42e7633844e0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2556,7 +2707,7 @@
     <x:mergeCell ref="A44:F44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08da6026d5b54c28"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ffbf0d02c764ea7"/>
 </x:worksheet>
 </file>
 
@@ -2692,13 +2843,13 @@
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
       <x:c r="A9" s="135" t="str">
-        <x:v>Trend of Vulnerabilities Discovered in Last 3 Months</x:v>
+        <x:v>Vulnerability Trend - Last 3 Months</x:v>
       </x:c>
       <x:c r="B9" s="136" t="str">
-        <x:v>Trend of Vulnerabilities Discovered in Last 3 Months</x:v>
+        <x:v>Vulnerability Trend - Last 3 Months</x:v>
       </x:c>
       <x:c r="C9" s="137" t="str">
-        <x:v>Trend of Vulnerabilities Discovered in Last 3 Months</x:v>
+        <x:v>Vulnerability Trend - Last 3 Months</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2708,6 +2859,9 @@
       <x:c r="B10" s="83" t="str">
         <x:v>Discovered</x:v>
       </x:c>
+      <x:c r="C10" s="83" t="str">
+        <x:v>Remediated</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="45" t="str">
@@ -2716,6 +2870,9 @@
       <x:c r="B11" s="45" t="n">
         <x:v>30</x:v>
       </x:c>
+      <x:c r="C11" s="45" t="n">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45" t="str">
@@ -2724,6 +2881,9 @@
       <x:c r="B12" s="45" t="n">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="C12" s="45" t="n">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45" t="str">
@@ -2731,6 +2891,9 @@
       </x:c>
       <x:c r="B13" s="45" t="n">
         <x:v>20</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="n">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="21" customHeight="1">
@@ -3070,7 +3233,7 @@
     <x:mergeCell ref="H27:L27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R951c3e55660a4891"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac7903cb3a6c4f35"/>
 </x:worksheet>
 </file>
 
@@ -3121,7 +3284,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="84" t="n">
-        <x:v>542</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B5" s="85" t="str"/>
       <x:c r="C5" s="86" t="str"/>
@@ -3180,13 +3343,13 @@
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="B12" s="45" t="n">
-        <x:v>98</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E12" s="49" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F12" s="45" t="n">
-        <x:v>123</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3194,13 +3357,13 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="B13" s="45" t="n">
-        <x:v>123</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E13" s="51" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="F13" s="45" t="n">
-        <x:v>419</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -3208,13 +3371,13 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="B14" s="45" t="n">
-        <x:v>148</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E14" s="53" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="F14" s="45" t="n">
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -3222,13 +3385,13 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="B15" s="45" t="n">
-        <x:v>173</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E15" s="55" t="str">
         <x:v>P4</x:v>
       </x:c>
       <x:c r="F15" s="45" t="n">
-        <x:v>0</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -3293,17 +3456,17 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="45" t="str">
-        <x:v>cs-asset-006.corp.example</x:v>
+        <x:v>cs-asset-021.corp.example</x:v>
       </x:c>
       <x:c r="B22" s="45" t="n">
-        <x:v>20</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C22" s="45" t="str"/>
       <x:c r="D22" s="45" t="str">
-        <x:v>cs-asset-006</x:v>
+        <x:v>cs-asset-021</x:v>
       </x:c>
       <x:c r="E22" s="45" t="n">
-        <x:v>20</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F22" s="45" t="str"/>
       <x:c r="G22" s="45" t="str"/>
@@ -3311,17 +3474,17 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="45" t="str">
-        <x:v>cs-asset-003.corp.example</x:v>
+        <x:v>cs-asset-022.corp.example</x:v>
       </x:c>
       <x:c r="B23" s="45" t="n">
-        <x:v>19</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C23" s="45" t="str"/>
       <x:c r="D23" s="45" t="str">
-        <x:v>cs-asset-003</x:v>
+        <x:v>cs-asset-022</x:v>
       </x:c>
       <x:c r="E23" s="45" t="n">
-        <x:v>19</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="45" t="str"/>
       <x:c r="G23" s="45" t="str"/>
@@ -3329,17 +3492,17 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="45" t="str">
-        <x:v>cs-asset-008.corp.example</x:v>
+        <x:v>cs-asset-023.corp.example</x:v>
       </x:c>
       <x:c r="B24" s="45" t="n">
-        <x:v>18</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C24" s="45" t="str"/>
       <x:c r="D24" s="45" t="str">
-        <x:v>cs-asset-008</x:v>
+        <x:v>cs-asset-023</x:v>
       </x:c>
       <x:c r="E24" s="45" t="n">
-        <x:v>18</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="45" t="str"/>
       <x:c r="G24" s="45" t="str"/>
@@ -3347,17 +3510,17 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="45" t="str">
-        <x:v>cs-asset-005.corp.example</x:v>
+        <x:v>cs-asset-024.corp.example</x:v>
       </x:c>
       <x:c r="B25" s="45" t="n">
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C25" s="45" t="str"/>
       <x:c r="D25" s="45" t="str">
-        <x:v>cs-asset-005</x:v>
+        <x:v>cs-asset-024</x:v>
       </x:c>
       <x:c r="E25" s="45" t="n">
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F25" s="45" t="str"/>
       <x:c r="G25" s="45" t="str"/>
@@ -3365,17 +3528,17 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="45" t="str">
-        <x:v>cs-asset-002.corp.example</x:v>
+        <x:v>cs-asset-025.corp.example</x:v>
       </x:c>
       <x:c r="B26" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="45" t="str"/>
       <x:c r="D26" s="45" t="str">
-        <x:v>cs-asset-002</x:v>
+        <x:v>cs-asset-025</x:v>
       </x:c>
       <x:c r="E26" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F26" s="45" t="str"/>
       <x:c r="G26" s="45" t="str"/>
@@ -3383,17 +3546,17 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="45" t="str">
-        <x:v>cs-asset-010.corp.example</x:v>
+        <x:v>cs-asset-026.corp.example</x:v>
       </x:c>
       <x:c r="B27" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C27" s="45" t="str"/>
       <x:c r="D27" s="45" t="str">
-        <x:v>cs-asset-010</x:v>
+        <x:v>cs-asset-026</x:v>
       </x:c>
       <x:c r="E27" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F27" s="45" t="str"/>
       <x:c r="G27" s="45" t="str"/>
@@ -3401,17 +3564,17 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="45" t="str">
-        <x:v>cs-asset-007.corp.example</x:v>
+        <x:v>cs-asset-027.corp.example</x:v>
       </x:c>
       <x:c r="B28" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C28" s="45" t="str"/>
       <x:c r="D28" s="45" t="str">
-        <x:v>cs-asset-007</x:v>
+        <x:v>cs-asset-027</x:v>
       </x:c>
       <x:c r="E28" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F28" s="45" t="str"/>
       <x:c r="G28" s="45" t="str"/>
@@ -3419,17 +3582,17 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="45" t="str">
-        <x:v>cs-asset-016.corp.example</x:v>
+        <x:v>cs-asset-028.corp.example</x:v>
       </x:c>
       <x:c r="B29" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C29" s="45" t="str"/>
       <x:c r="D29" s="45" t="str">
-        <x:v>cs-asset-016</x:v>
+        <x:v>cs-asset-028</x:v>
       </x:c>
       <x:c r="E29" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F29" s="45" t="str"/>
       <x:c r="G29" s="45" t="str"/>
@@ -3437,17 +3600,17 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="45" t="str">
-        <x:v>cs-asset-024.corp.example</x:v>
+        <x:v>cs-asset-029.corp.example</x:v>
       </x:c>
       <x:c r="B30" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C30" s="45" t="str"/>
       <x:c r="D30" s="45" t="str">
-        <x:v>cs-asset-024</x:v>
+        <x:v>cs-asset-029</x:v>
       </x:c>
       <x:c r="E30" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F30" s="45" t="str"/>
       <x:c r="G30" s="45" t="str"/>
@@ -3455,17 +3618,17 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="45" t="str">
-        <x:v>cs-asset-032.corp.example</x:v>
+        <x:v>cs-asset-030.corp.example</x:v>
       </x:c>
       <x:c r="B31" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C31" s="45" t="str"/>
       <x:c r="D31" s="45" t="str">
-        <x:v>cs-asset-032</x:v>
+        <x:v>cs-asset-030</x:v>
       </x:c>
       <x:c r="E31" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F31" s="45" t="str"/>
       <x:c r="G31" s="45" t="str"/>
@@ -3483,6 +3646,6 @@
     <x:mergeCell ref="A20:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra752c271b1694709"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7372905713354a5b"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize unified reporting workflows (#8)
Co-authored-by: Mohammed Shahid <DrHayabusa@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/final/Excel/MVA_CrowdStrike_Final_Report.xlsx
+++ b/final/Excel/MVA_CrowdStrike_Final_Report.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R674dcd0a08cc4d7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="Rb7e7139243e44fcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="Rf1fd88f624104ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="Rf5819292cd5d4633"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="R04534b11f3254dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="R2f3a99e5239f49be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1377,7 +1377,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Discovered Vulnerabilities - Last 3 Months</a:t>
+              <a:t>Vulnerabilities Discovered</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1487,6 +1487,127 @@
 </file>
 
 <file path=xl/drawings/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>Vulnerabilities Remediated</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Remediated</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="70AD47"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Monthly Dashboard'!$A$11:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Monthly Dashboard'!$C$11:$C$13</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="30"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1629,7 +1750,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2a8519470dd402f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5a58a256c6be4a33"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1659,7 +1780,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R37188d9774c84e6b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b69d487e8fd429f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1689,7 +1810,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdac270d4f4fd44af"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R95c39958b6394b58"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1702,13 +1823,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1724,7 +1845,37 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6586b49a59e4dfe"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R180c710a43e74686"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rae89106a3a7e447a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1759,7 +1910,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb5ef71c409e4b7a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R207f42e7633844e0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2556,7 +2707,7 @@
     <x:mergeCell ref="A44:F44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08da6026d5b54c28"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ffbf0d02c764ea7"/>
 </x:worksheet>
 </file>
 
@@ -2692,13 +2843,13 @@
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
       <x:c r="A9" s="135" t="str">
-        <x:v>Trend of Vulnerabilities Discovered in Last 3 Months</x:v>
+        <x:v>Vulnerability Trend - Last 3 Months</x:v>
       </x:c>
       <x:c r="B9" s="136" t="str">
-        <x:v>Trend of Vulnerabilities Discovered in Last 3 Months</x:v>
+        <x:v>Vulnerability Trend - Last 3 Months</x:v>
       </x:c>
       <x:c r="C9" s="137" t="str">
-        <x:v>Trend of Vulnerabilities Discovered in Last 3 Months</x:v>
+        <x:v>Vulnerability Trend - Last 3 Months</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2708,6 +2859,9 @@
       <x:c r="B10" s="83" t="str">
         <x:v>Discovered</x:v>
       </x:c>
+      <x:c r="C10" s="83" t="str">
+        <x:v>Remediated</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="45" t="str">
@@ -2716,6 +2870,9 @@
       <x:c r="B11" s="45" t="n">
         <x:v>30</x:v>
       </x:c>
+      <x:c r="C11" s="45" t="n">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45" t="str">
@@ -2724,6 +2881,9 @@
       <x:c r="B12" s="45" t="n">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="C12" s="45" t="n">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45" t="str">
@@ -2731,6 +2891,9 @@
       </x:c>
       <x:c r="B13" s="45" t="n">
         <x:v>20</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="n">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="21" customHeight="1">
@@ -3070,7 +3233,7 @@
     <x:mergeCell ref="H27:L27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R951c3e55660a4891"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac7903cb3a6c4f35"/>
 </x:worksheet>
 </file>
 
@@ -3121,7 +3284,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="84" t="n">
-        <x:v>542</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B5" s="85" t="str"/>
       <x:c r="C5" s="86" t="str"/>
@@ -3180,13 +3343,13 @@
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="B12" s="45" t="n">
-        <x:v>98</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E12" s="49" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F12" s="45" t="n">
-        <x:v>123</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3194,13 +3357,13 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="B13" s="45" t="n">
-        <x:v>123</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E13" s="51" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="F13" s="45" t="n">
-        <x:v>419</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -3208,13 +3371,13 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="B14" s="45" t="n">
-        <x:v>148</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E14" s="53" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="F14" s="45" t="n">
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -3222,13 +3385,13 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="B15" s="45" t="n">
-        <x:v>173</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E15" s="55" t="str">
         <x:v>P4</x:v>
       </x:c>
       <x:c r="F15" s="45" t="n">
-        <x:v>0</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -3293,17 +3456,17 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="45" t="str">
-        <x:v>cs-asset-006.corp.example</x:v>
+        <x:v>cs-asset-021.corp.example</x:v>
       </x:c>
       <x:c r="B22" s="45" t="n">
-        <x:v>20</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C22" s="45" t="str"/>
       <x:c r="D22" s="45" t="str">
-        <x:v>cs-asset-006</x:v>
+        <x:v>cs-asset-021</x:v>
       </x:c>
       <x:c r="E22" s="45" t="n">
-        <x:v>20</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F22" s="45" t="str"/>
       <x:c r="G22" s="45" t="str"/>
@@ -3311,17 +3474,17 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="45" t="str">
-        <x:v>cs-asset-003.corp.example</x:v>
+        <x:v>cs-asset-022.corp.example</x:v>
       </x:c>
       <x:c r="B23" s="45" t="n">
-        <x:v>19</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C23" s="45" t="str"/>
       <x:c r="D23" s="45" t="str">
-        <x:v>cs-asset-003</x:v>
+        <x:v>cs-asset-022</x:v>
       </x:c>
       <x:c r="E23" s="45" t="n">
-        <x:v>19</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="45" t="str"/>
       <x:c r="G23" s="45" t="str"/>
@@ -3329,17 +3492,17 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="45" t="str">
-        <x:v>cs-asset-008.corp.example</x:v>
+        <x:v>cs-asset-023.corp.example</x:v>
       </x:c>
       <x:c r="B24" s="45" t="n">
-        <x:v>18</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C24" s="45" t="str"/>
       <x:c r="D24" s="45" t="str">
-        <x:v>cs-asset-008</x:v>
+        <x:v>cs-asset-023</x:v>
       </x:c>
       <x:c r="E24" s="45" t="n">
-        <x:v>18</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="45" t="str"/>
       <x:c r="G24" s="45" t="str"/>
@@ -3347,17 +3510,17 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="45" t="str">
-        <x:v>cs-asset-005.corp.example</x:v>
+        <x:v>cs-asset-024.corp.example</x:v>
       </x:c>
       <x:c r="B25" s="45" t="n">
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C25" s="45" t="str"/>
       <x:c r="D25" s="45" t="str">
-        <x:v>cs-asset-005</x:v>
+        <x:v>cs-asset-024</x:v>
       </x:c>
       <x:c r="E25" s="45" t="n">
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F25" s="45" t="str"/>
       <x:c r="G25" s="45" t="str"/>
@@ -3365,17 +3528,17 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="45" t="str">
-        <x:v>cs-asset-002.corp.example</x:v>
+        <x:v>cs-asset-025.corp.example</x:v>
       </x:c>
       <x:c r="B26" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="45" t="str"/>
       <x:c r="D26" s="45" t="str">
-        <x:v>cs-asset-002</x:v>
+        <x:v>cs-asset-025</x:v>
       </x:c>
       <x:c r="E26" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F26" s="45" t="str"/>
       <x:c r="G26" s="45" t="str"/>
@@ -3383,17 +3546,17 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="45" t="str">
-        <x:v>cs-asset-010.corp.example</x:v>
+        <x:v>cs-asset-026.corp.example</x:v>
       </x:c>
       <x:c r="B27" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C27" s="45" t="str"/>
       <x:c r="D27" s="45" t="str">
-        <x:v>cs-asset-010</x:v>
+        <x:v>cs-asset-026</x:v>
       </x:c>
       <x:c r="E27" s="45" t="n">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F27" s="45" t="str"/>
       <x:c r="G27" s="45" t="str"/>
@@ -3401,17 +3564,17 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="45" t="str">
-        <x:v>cs-asset-007.corp.example</x:v>
+        <x:v>cs-asset-027.corp.example</x:v>
       </x:c>
       <x:c r="B28" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C28" s="45" t="str"/>
       <x:c r="D28" s="45" t="str">
-        <x:v>cs-asset-007</x:v>
+        <x:v>cs-asset-027</x:v>
       </x:c>
       <x:c r="E28" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F28" s="45" t="str"/>
       <x:c r="G28" s="45" t="str"/>
@@ -3419,17 +3582,17 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="45" t="str">
-        <x:v>cs-asset-016.corp.example</x:v>
+        <x:v>cs-asset-028.corp.example</x:v>
       </x:c>
       <x:c r="B29" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C29" s="45" t="str"/>
       <x:c r="D29" s="45" t="str">
-        <x:v>cs-asset-016</x:v>
+        <x:v>cs-asset-028</x:v>
       </x:c>
       <x:c r="E29" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F29" s="45" t="str"/>
       <x:c r="G29" s="45" t="str"/>
@@ -3437,17 +3600,17 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="45" t="str">
-        <x:v>cs-asset-024.corp.example</x:v>
+        <x:v>cs-asset-029.corp.example</x:v>
       </x:c>
       <x:c r="B30" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C30" s="45" t="str"/>
       <x:c r="D30" s="45" t="str">
-        <x:v>cs-asset-024</x:v>
+        <x:v>cs-asset-029</x:v>
       </x:c>
       <x:c r="E30" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F30" s="45" t="str"/>
       <x:c r="G30" s="45" t="str"/>
@@ -3455,17 +3618,17 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="45" t="str">
-        <x:v>cs-asset-032.corp.example</x:v>
+        <x:v>cs-asset-030.corp.example</x:v>
       </x:c>
       <x:c r="B31" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C31" s="45" t="str"/>
       <x:c r="D31" s="45" t="str">
-        <x:v>cs-asset-032</x:v>
+        <x:v>cs-asset-030</x:v>
       </x:c>
       <x:c r="E31" s="45" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F31" s="45" t="str"/>
       <x:c r="G31" s="45" t="str"/>
@@ -3483,6 +3646,6 @@
     <x:mergeCell ref="A20:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra752c271b1694709"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7372905713354a5b"/>
 </x:worksheet>
 </file>
</xml_diff>